<commit_message>
Updated HCAI in hospitals summary
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Room Accommodation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC227465-16CF-4C79-8119-0FC726867653}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B98D5B2-710A-45A7-9598-4A6BF11AA6E7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="3792" yWindow="1728" windowWidth="19164" windowHeight="10944" activeTab="1" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -579,6 +579,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -591,7 +592,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -959,23 +959,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.6796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.40625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.40625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.40625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="83.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="164.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="83.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="164.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="2" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1045,11 +1045,11 @@
       <c r="K2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="32" t="s">
+      <c r="L2" s="28" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="3" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1083,11 +1083,11 @@
       <c r="K3" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="32" t="s">
+      <c r="L3" s="28" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="4" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="5" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A5" s="17">
         <v>4</v>
       </c>
@@ -1157,11 +1157,11 @@
       <c r="K5" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="L5" s="32" t="s">
+      <c r="L5" s="28" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="6" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A6" s="17">
         <v>5</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="7" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A7" s="17">
         <v>6</v>
       </c>
@@ -1233,11 +1233,11 @@
       <c r="K7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="32" t="s">
+      <c r="L7" s="28" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="8" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A8" s="17">
         <v>7</v>
       </c>
@@ -1271,11 +1271,11 @@
       <c r="K8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="32" t="s">
+      <c r="L8" s="28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1305,11 +1305,11 @@
       <c r="K9" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="32" t="s">
+      <c r="L9" s="28" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="10" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="11" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="12" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -1398,14 +1398,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:M14"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.6328125" customWidth="1"/>
-    <col min="3" max="10" width="12.40625" customWidth="1"/>
-    <col min="13" max="13" width="16.76953125" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="10" width="12.44140625" customWidth="1"/>
+    <col min="13" max="13" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.75">
+    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1431,26 +1431,26 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.75">
-      <c r="B2" s="30" t="s">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B2" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="30"/>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:13" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
-      <c r="B3" s="31"/>
+    <row r="3" spans="2:13" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B3" s="32"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
       </c>
@@ -1479,7 +1479,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
         <v>46</v>
       </c>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
         <v>45</v>
       </c>
@@ -1527,7 +1527,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="5">
         <v>2</v>
@@ -1539,7 +1539,7 @@
         <v>2</v>
       </c>
       <c r="J5" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5" s="11"/>
       <c r="L5" s="13"/>
@@ -1547,7 +1547,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="6" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
         <v>44</v>
       </c>
@@ -1581,7 +1581,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="7" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>43</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="8" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
         <v>42</v>
       </c>
@@ -1647,7 +1647,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="9" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
         <v>41</v>
       </c>
@@ -1679,7 +1679,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
         <v>40</v>
       </c>
@@ -1711,7 +1711,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="11" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
         <v>39</v>
       </c>
@@ -1743,7 +1743,7 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="12" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
         <v>38</v>
       </c>
@@ -1775,7 +1775,7 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="13" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="6" t="s">
         <v>37</v>
       </c>
@@ -1807,7 +1807,7 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="14" spans="2:13" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
Minor changes and additions to hospital site and indicator spreadsheets.
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC227465-16CF-4C79-8119-0FC726867653}"/>
+  <xr:revisionPtr revIDLastSave="239" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{035CE1EE-8418-4C19-9CAA-0900FDBDF8DE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="-28920" yWindow="10620" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="79">
   <si>
     <t>num</t>
   </si>
@@ -265,6 +265,15 @@
   </si>
   <si>
     <t>One ward only, 20 of 28 beds SR. Currently used as interim beds for RAAC remedial work.</t>
+  </si>
+  <si>
+    <t>Cleaning Staff WTE</t>
+  </si>
+  <si>
+    <t>James Paget (concept)*</t>
+  </si>
+  <si>
+    <t>* Note re: fucntion fo the ward not suitable for stuyd</t>
   </si>
 </sst>
 </file>
@@ -518,7 +527,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -579,6 +588,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -591,7 +601,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1045,7 +1060,7 @@
       <c r="K2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="32" t="s">
+      <c r="L2" s="28" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1083,7 +1098,7 @@
       <c r="K3" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="32" t="s">
+      <c r="L3" s="28" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1157,7 +1172,7 @@
       <c r="K5" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="L5" s="32" t="s">
+      <c r="L5" s="28" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1233,7 +1248,7 @@
       <c r="K7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="32" t="s">
+      <c r="L7" s="28" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1271,7 +1286,7 @@
       <c r="K8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="32" t="s">
+      <c r="L8" s="28" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1305,7 +1320,7 @@
       <c r="K9" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="32" t="s">
+      <c r="L9" s="28" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1397,7 +1412,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
-  <dimension ref="B1:M14"/>
+  <dimension ref="B1:N17"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="2" max="2" width="16.6328125" customWidth="1"/>
@@ -1405,7 +1420,7 @@
     <col min="13" max="13" width="16.76953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.75">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.75">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1431,26 +1446,26 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.75">
-      <c r="B2" s="30" t="s">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.75">
+      <c r="B2" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="30"/>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:13" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
-      <c r="B3" s="31"/>
+    <row r="3" spans="2:14" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="B3" s="32"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
       </c>
@@ -1464,7 +1479,7 @@
         <v>19</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>13</v>
@@ -1479,7 +1494,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B4" s="6" t="s">
         <v>46</v>
       </c>
@@ -1499,7 +1514,7 @@
         <v>2</v>
       </c>
       <c r="H4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="5">
         <v>0</v>
@@ -1513,7 +1528,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B5" s="6" t="s">
         <v>45</v>
       </c>
@@ -1546,8 +1561,11 @@
       <c r="M5" s="14" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="6" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="N5" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B6" s="6" t="s">
         <v>44</v>
       </c>
@@ -1580,8 +1598,11 @@
       <c r="M6" s="12" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="7" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="N6" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B7" s="6" t="s">
         <v>43</v>
       </c>
@@ -1614,8 +1635,11 @@
       <c r="M7" s="12" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="8" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="N7" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B8" s="6" t="s">
         <v>42</v>
       </c>
@@ -1647,7 +1671,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="9" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B9" s="6" t="s">
         <v>41</v>
       </c>
@@ -1679,7 +1703,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B10" s="6" t="s">
         <v>40</v>
       </c>
@@ -1711,7 +1735,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="11" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B11" s="6" t="s">
         <v>39</v>
       </c>
@@ -1743,12 +1767,12 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="12" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B12" s="6" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="C12" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="5">
         <v>1</v>
@@ -1757,27 +1781,23 @@
         <v>1</v>
       </c>
       <c r="F12" s="5">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G12" s="5"/>
       <c r="H12" s="5">
         <v>1</v>
       </c>
       <c r="I12" s="5">
         <v>2</v>
       </c>
-      <c r="J12" s="4">
-        <v>0</v>
-      </c>
+      <c r="J12" s="4"/>
       <c r="K12" s="11"/>
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="13" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B13" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C13" s="5">
         <v>1</v>
@@ -1807,44 +1827,81 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:13" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="B14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="2">
-        <v>1</v>
-      </c>
-      <c r="D14" s="2">
-        <v>1</v>
-      </c>
-      <c r="E14" s="2">
-        <v>1</v>
-      </c>
-      <c r="F14" s="2">
+    <row r="14" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="B14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="5">
+        <v>1</v>
+      </c>
+      <c r="D14" s="5">
+        <v>1</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1</v>
+      </c>
+      <c r="F14" s="5">
         <v>0</v>
       </c>
-      <c r="G14" s="2">
-        <v>2</v>
-      </c>
-      <c r="H14" s="2">
-        <v>1</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0</v>
-      </c>
-      <c r="J14" s="1">
+      <c r="G14" s="5">
+        <v>2</v>
+      </c>
+      <c r="H14" s="5">
+        <v>1</v>
+      </c>
+      <c r="I14" s="5">
+        <v>2</v>
+      </c>
+      <c r="J14" s="4">
         <v>0</v>
       </c>
       <c r="K14" s="11"/>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
+    </row>
+    <row r="15" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="B15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>2</v>
+      </c>
+      <c r="H15" s="2">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0</v>
+      </c>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+    </row>
+    <row r="17" spans="2:2" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="B17" s="34" t="s">
+        <v>78</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C2:J2"/>
     <mergeCell ref="B2:B3"/>
   </mergeCells>
-  <conditionalFormatting sqref="C4:J14">
+  <conditionalFormatting sqref="C4:J15">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>2</formula>
     </cfRule>

</xml_diff>

<commit_message>
updates to ods codes for sites pre and post change
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="243" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{957D9F4F-676E-45CA-8076-4C5891B4AE67}"/>
+  <xr:revisionPtr revIDLastSave="252" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A62245F6-AA4A-493A-98DB-FFBBFB497F71}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="10620" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="81">
   <si>
     <t>num</t>
   </si>
@@ -268,6 +268,18 @@
   </si>
   <si>
     <t>Cleaning Staff WTE</t>
+  </si>
+  <si>
+    <t>RGM22</t>
+  </si>
+  <si>
+    <t>RALC7+RG9C7+RVLC7</t>
+  </si>
+  <si>
+    <t>REMRQ+RQ617</t>
+  </si>
+  <si>
+    <t>RGN42+RQQ10</t>
   </si>
 </sst>
 </file>
@@ -979,8 +991,8 @@
     <col min="7" max="7" width="8.1328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.40625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="83.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6796875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="164.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1049,7 +1061,7 @@
       </c>
       <c r="I2" s="17"/>
       <c r="J2" s="17" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="K2" s="17" t="s">
         <v>6</v>
@@ -1087,10 +1099,10 @@
         <v>67</v>
       </c>
       <c r="J3" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" s="17" t="s">
         <v>54</v>
-      </c>
-      <c r="K3" s="17" t="s">
-        <v>12</v>
       </c>
       <c r="L3" s="28" t="s">
         <v>71</v>
@@ -1128,7 +1140,7 @@
         <v>53</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="L4" s="17" t="s">
         <v>69</v>
@@ -1164,7 +1176,7 @@
         <v>66</v>
       </c>
       <c r="K5" s="17" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="L5" s="28" t="s">
         <v>31</v>
@@ -1199,7 +1211,7 @@
         <v>60</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="K6" s="17" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Update site codes in summary hosp file. Add monthly inpatient data. Add script with functions.
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="252" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A62245F6-AA4A-493A-98DB-FFBBFB497F71}"/>
+  <xr:revisionPtr revIDLastSave="253" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F43A29C-EE64-4355-810A-CCEAEB8537F1}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="35" yWindow="5310" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -980,23 +980,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.40625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.40625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.40625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="83.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.90625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.6796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="164.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39" customWidth="1"/>
+    <col min="10" max="10" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="164.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1034,7 +1034,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="2" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1070,7 +1070,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="3" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="4" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="5" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="17">
         <v>4</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="6" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="17">
         <v>5</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="17">
         <v>6</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="8" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="17">
         <v>7</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="10" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="11" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="12" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -1419,14 +1419,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:N17"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.6328125" customWidth="1"/>
-    <col min="3" max="10" width="12.40625" customWidth="1"/>
-    <col min="13" max="13" width="16.76953125" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
+    <col min="3" max="10" width="12.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.75">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
         <v>48</v>
       </c>
@@ -1470,7 +1470,7 @@
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:14" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:14" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="B3" s="34"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
@@ -1500,7 +1500,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="6" t="s">
         <v>46</v>
       </c>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
         <v>45</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="6" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
         <v>44</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="7" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
         <v>43</v>
       </c>
@@ -1645,7 +1645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="8" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
         <v>42</v>
       </c>
@@ -1677,7 +1677,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="9" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
         <v>41</v>
       </c>
@@ -1709,7 +1709,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
         <v>40</v>
       </c>
@@ -1741,7 +1741,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="11" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
         <v>39</v>
       </c>
@@ -1773,7 +1773,7 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="12" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6" t="s">
         <v>76</v>
       </c>
@@ -1801,7 +1801,7 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="13" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
         <v>38</v>
       </c>
@@ -1833,7 +1833,7 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="14" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6" t="s">
         <v>37</v>
       </c>
@@ -1865,7 +1865,7 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="2:14" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="15" spans="2:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
@@ -1897,7 +1897,7 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.75">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="30"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated pre and post site codes based on SUS activity
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Room Accommodation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="262" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFA5A02C-6A89-4145-933A-C2AA19F81372}"/>
+  <xr:revisionPtr revIDLastSave="279" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0103418E-A856-4F5D-A194-4F2CBF1A312E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="1" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
   <si>
     <t>num</t>
   </si>
@@ -57,9 +57,6 @@
     <t>Liverpool</t>
   </si>
   <si>
-    <t>REMRQ</t>
-  </si>
-  <si>
     <t>Royal Papworth</t>
   </si>
   <si>
@@ -93,18 +90,12 @@
     <t>Bristol</t>
   </si>
   <si>
-    <t>RVJ01</t>
-  </si>
-  <si>
     <t>Tunbridge Wells</t>
   </si>
   <si>
     <t>Kent</t>
   </si>
   <si>
-    <t>RWFTW</t>
-  </si>
-  <si>
     <t>Ulster Hospital</t>
   </si>
   <si>
@@ -195,12 +186,6 @@
     <t>No data prior to SBR change</t>
   </si>
   <si>
-    <t>RGM21</t>
-  </si>
-  <si>
-    <t>REN20</t>
-  </si>
-  <si>
     <t>Tertiary cardio-thoracic centre.</t>
   </si>
   <si>
@@ -216,9 +201,6 @@
     <t>post_all</t>
   </si>
   <si>
-    <t>Surgical wards only</t>
-  </si>
-  <si>
     <t>weblink_info</t>
   </si>
   <si>
@@ -228,15 +210,9 @@
     <t>ods_code_post</t>
   </si>
   <si>
-    <t>RWF01+RWF02</t>
-  </si>
-  <si>
     <t>Peterborough (district) Hospital</t>
   </si>
   <si>
-    <t>RGN42</t>
-  </si>
-  <si>
     <t>Day case and routine inpatient only?</t>
   </si>
   <si>
@@ -255,9 +231,6 @@
     <t>Jan 11 for W&amp;C, Sep 11 for remainder of inpatient. Two sites closed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Trust info - 75% (of 800 brunel) are single bed rooms. </t>
-  </si>
-  <si>
     <t>http://www.leaderflushshapland.co.uk/Project-gallery/Southmead-Hospital; https://api.cqc.org.uk/public/v1/reports/d43a3164-270b-4213-b3db-50790b1f4a6d?20210121222525</t>
   </si>
   <si>
@@ -267,22 +240,31 @@
     <t>Cleaning Staff WTE</t>
   </si>
   <si>
-    <t>RGM22</t>
-  </si>
-  <si>
-    <t>RALC7+RG9C7+RVLC7</t>
-  </si>
-  <si>
     <t>REMRQ+RQ617</t>
   </si>
   <si>
-    <t>RGN42+RQQ10</t>
-  </si>
-  <si>
     <t>HCAI*</t>
   </si>
   <si>
     <t>*Marked according to being able to do a composite measure. Could potentially look at cdiff only for Chase Farm and Southmead</t>
+  </si>
+  <si>
+    <t>RGM21+RGM22</t>
+  </si>
+  <si>
+    <t>RGN42+RGN80</t>
+  </si>
+  <si>
+    <t>Planned surgery, select specialties</t>
+  </si>
+  <si>
+    <t>RVJ01+RVY20</t>
+  </si>
+  <si>
+    <t>Trust info - 75% (of 800 brunel) are single bed rooms. Merger of Frenchay &amp; Southmead</t>
+  </si>
+  <si>
+    <t>RWF01+RWF02+RWFTW</t>
   </si>
 </sst>
 </file>
@@ -983,23 +965,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" customWidth="1"/>
-    <col min="10" max="10" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="164.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="23.1328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="164.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1013,31 +994,31 @@
         <v>3</v>
       </c>
       <c r="E1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="K1" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="G1" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="I1" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="J1" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="K1" s="17" t="s">
-        <v>62</v>
-      </c>
       <c r="L1" s="17" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1064,21 +1045,21 @@
       </c>
       <c r="I2" s="17"/>
       <c r="J2" s="17" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>6</v>
+        <v>67</v>
       </c>
       <c r="L2" s="28" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A3" s="17">
         <v>2</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>5</v>
@@ -1099,27 +1080,27 @@
         <v>89</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="L3" s="28" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A4" s="17">
         <v>3</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>7</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>8</v>
       </c>
       <c r="D4" s="18">
         <v>43586</v>
@@ -1137,27 +1118,27 @@
         <v>237</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A5" s="17">
         <v>4</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="18">
         <v>40483</v>
@@ -1176,24 +1157,24 @@
       </c>
       <c r="I5" s="17"/>
       <c r="J5" s="17" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="K5" s="17" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="L5" s="28" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A6" s="17">
         <v>5</v>
       </c>
       <c r="B6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>13</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>14</v>
       </c>
       <c r="D6" s="18">
         <v>43344</v>
@@ -1211,27 +1192,27 @@
         <v>50</v>
       </c>
       <c r="I6" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="L6" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="J6" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="K6" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="17" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A7" s="17">
         <v>6</v>
       </c>
       <c r="B7" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>16</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>17</v>
       </c>
       <c r="D7" s="18">
         <v>41760</v>
@@ -1249,27 +1230,27 @@
         <v>800</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="K7" s="17" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="L7" s="28" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A8" s="17">
         <v>7</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8" s="18">
         <v>40544</v>
@@ -1287,27 +1268,27 @@
         <v>503</v>
       </c>
       <c r="I8" s="17" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="L8" s="28" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.8" x14ac:dyDescent="0.4">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A9" s="24">
         <v>8</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D9" s="25">
         <v>45047</v>
@@ -1321,27 +1302,27 @@
       </c>
       <c r="H9" s="26"/>
       <c r="I9" s="24" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="L9" s="28" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A10" s="20">
         <v>9</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D10" s="21">
         <v>42826</v>
@@ -1353,19 +1334,19 @@
       <c r="I10" s="17"/>
       <c r="J10" s="17"/>
       <c r="K10" s="17" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A11" s="20">
         <v>10</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D11" s="21">
         <v>42095</v>
@@ -1377,19 +1358,19 @@
       <c r="I11" s="17"/>
       <c r="J11" s="17"/>
       <c r="K11" s="17" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A12" s="20">
         <v>11</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D12" s="21">
         <v>44136</v>
@@ -1401,7 +1382,7 @@
       <c r="I12" s="17"/>
       <c r="J12" s="17"/>
       <c r="K12" s="17" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L12" s="17"/>
     </row>
@@ -1422,14 +1403,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:P17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="10" width="12.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" customWidth="1"/>
+    <col min="3" max="10" width="12.453125" customWidth="1"/>
+    <col min="13" max="13" width="16.6796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.75">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1455,12 +1436,12 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.75">
       <c r="B2" s="33" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C2" s="31" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D2" s="31"/>
       <c r="E2" s="31"/>
@@ -1473,39 +1454,39 @@
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:16" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:16" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
       <c r="B3" s="34"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B4" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C4" s="5">
         <v>1</v>
@@ -1533,13 +1514,13 @@
       </c>
       <c r="K4" s="11"/>
       <c r="L4" s="11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B5" s="6" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="C5" s="5">
         <v>1</v>
@@ -1568,18 +1549,18 @@
       <c r="K5" s="11"/>
       <c r="L5" s="13"/>
       <c r="M5" s="14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="N5" s="29">
         <v>1</v>
       </c>
       <c r="P5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="6" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B6" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C6" s="5">
         <v>1</v>
@@ -1608,15 +1589,15 @@
       <c r="K6" s="11"/>
       <c r="L6" s="16"/>
       <c r="M6" s="12" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="N6" s="29">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B7" s="6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C7" s="5">
         <v>1</v>
@@ -1645,15 +1626,15 @@
       <c r="K7" s="11"/>
       <c r="L7" s="15"/>
       <c r="M7" s="12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="N7" s="29">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B8" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C8" s="5">
         <v>1</v>
@@ -1683,9 +1664,9 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B9" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C9" s="5">
         <v>1</v>
@@ -1715,9 +1696,9 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B10" s="6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C10" s="5">
         <v>1</v>
@@ -1747,9 +1728,9 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B11" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C11" s="5">
         <v>1</v>
@@ -1779,9 +1760,9 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B12" s="6" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
@@ -1807,9 +1788,9 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B13" s="6" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C13" s="5">
         <v>1</v>
@@ -1839,9 +1820,9 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B14" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C14" s="5">
         <v>1</v>
@@ -1871,9 +1852,9 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B15" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C15" s="2">
         <v>1</v>
@@ -1903,7 +1884,7 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.75">
       <c r="B17" s="30"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add reference tables of cancer and cardiac centres for control site filtering
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="279" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0103418E-A856-4F5D-A194-4F2CBF1A312E}"/>
+  <xr:revisionPtr revIDLastSave="281" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5507A48-8FA8-4EDB-9120-880B9605602A}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="-28920" yWindow="10620" windowWidth="29040" windowHeight="15840" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -258,13 +258,13 @@
     <t>Planned surgery, select specialties</t>
   </si>
   <si>
-    <t>RVJ01+RVY20</t>
-  </si>
-  <si>
     <t>Trust info - 75% (of 800 brunel) are single bed rooms. Merger of Frenchay &amp; Southmead</t>
   </si>
   <si>
     <t>RWF01+RWF02+RWFTW</t>
+  </si>
+  <si>
+    <t>RVJ01+RVJ20</t>
   </si>
 </sst>
 </file>
@@ -965,10 +965,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.6796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
@@ -976,11 +976,11 @@
     <col min="7" max="7" width="8.08984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" customWidth="1"/>
-    <col min="10" max="11" width="23.1328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="23.08984375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="164.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="2" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="3" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="4" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="5" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="17">
         <v>4</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="6" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="17">
         <v>5</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="17">
         <v>6</v>
       </c>
@@ -1230,19 +1230,19 @@
         <v>800</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K7" s="17" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L7" s="28" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="8" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="17">
         <v>7</v>
       </c>
@@ -1271,16 +1271,16 @@
         <v>63</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L8" s="28" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="10" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="11" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="12" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -1403,14 +1403,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:P17"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.54296875" customWidth="1"/>
     <col min="3" max="10" width="12.453125" customWidth="1"/>
-    <col min="13" max="13" width="16.6796875" customWidth="1"/>
+    <col min="13" max="13" width="16.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.75">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B2" s="33" t="s">
         <v>44</v>
       </c>
@@ -1454,7 +1454,7 @@
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:16" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:16" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B3" s="34"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
@@ -1484,7 +1484,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="6" t="s">
         <v>42</v>
       </c>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>68</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>40</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
@@ -1664,7 +1664,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>38</v>
       </c>
@@ -1696,7 +1696,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>37</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>36</v>
       </c>
@@ -1760,7 +1760,7 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>66</v>
       </c>
@@ -1788,7 +1788,7 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>35</v>
       </c>
@@ -1820,7 +1820,7 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>34</v>
       </c>
@@ -1852,7 +1852,7 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>33</v>
       </c>
@@ -1884,7 +1884,7 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.75">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="30"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating staff turnover indicator
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Room Accommodation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="281" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5507A48-8FA8-4EDB-9120-880B9605602A}"/>
+  <xr:revisionPtr revIDLastSave="285" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{410FC904-7771-4E09-822C-AC205C32145E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="10620" windowWidth="29040" windowHeight="15840" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="1128" yWindow="0" windowWidth="21912" windowHeight="13800" activeTab="1" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -965,22 +965,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" customWidth="1"/>
-    <col min="10" max="11" width="23.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="164.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="164.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A5" s="17">
         <v>4</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A6" s="17">
         <v>5</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A7" s="17">
         <v>6</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A8" s="17">
         <v>7</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -1403,14 +1403,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:P17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.54296875" customWidth="1"/>
-    <col min="3" max="10" width="12.453125" customWidth="1"/>
-    <col min="13" max="13" width="16.6328125" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="10" width="12.44140625" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B2" s="33" t="s">
         <v>44</v>
       </c>
@@ -1454,7 +1454,7 @@
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:16" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:16" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B3" s="34"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
@@ -1484,7 +1484,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
         <v>42</v>
       </c>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
         <v>68</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>40</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
@@ -1664,7 +1664,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
         <v>38</v>
       </c>
@@ -1696,7 +1696,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
         <v>37</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
         <v>36</v>
       </c>
@@ -1760,7 +1760,7 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
         <v>66</v>
       </c>
@@ -1788,7 +1788,7 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="6" t="s">
         <v>35</v>
       </c>
@@ -1820,7 +1820,7 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="6" t="s">
         <v>34</v>
       </c>
@@ -1831,7 +1831,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="5">
         <v>0</v>
@@ -1840,10 +1840,10 @@
         <v>2</v>
       </c>
       <c r="H14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J14" s="4">
         <v>0</v>
@@ -1852,7 +1852,7 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>33</v>
       </c>
@@ -1884,7 +1884,7 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="30"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
no changes to file made (O365 autosave of accidental and reveresed cell change) but thinks there are so pushing for cleanliness...
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Room Accommodation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="285" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{410FC904-7771-4E09-822C-AC205C32145E}"/>
   <bookViews>
-    <workbookView xWindow="1128" yWindow="0" windowWidth="21912" windowHeight="13800" activeTab="1" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -965,22 +965,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" customWidth="1"/>
-    <col min="10" max="11" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="164.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="164.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A5" s="17">
         <v>4</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A6" s="17">
         <v>5</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A7" s="17">
         <v>6</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A8" s="17">
         <v>7</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -1403,14 +1403,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:P17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="10" width="12.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" customWidth="1"/>
+    <col min="3" max="10" width="12.453125" customWidth="1"/>
+    <col min="13" max="13" width="16.6796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.75">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.75">
       <c r="B2" s="33" t="s">
         <v>44</v>
       </c>
@@ -1454,7 +1454,7 @@
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:16" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:16" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
       <c r="B3" s="34"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
@@ -1484,7 +1484,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B4" s="6" t="s">
         <v>42</v>
       </c>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B5" s="6" t="s">
         <v>68</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B7" s="6" t="s">
         <v>40</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
@@ -1664,7 +1664,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B9" s="6" t="s">
         <v>38</v>
       </c>
@@ -1696,7 +1696,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B10" s="6" t="s">
         <v>37</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B11" s="6" t="s">
         <v>36</v>
       </c>
@@ -1760,7 +1760,7 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B12" s="6" t="s">
         <v>66</v>
       </c>
@@ -1788,7 +1788,7 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B13" s="6" t="s">
         <v>35</v>
       </c>
@@ -1820,7 +1820,7 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B14" s="6" t="s">
         <v>34</v>
       </c>
@@ -1852,7 +1852,7 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B15" s="3" t="s">
         <v>33</v>
       </c>
@@ -1884,7 +1884,7 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.75">
       <c r="B17" s="30"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added sbr % plots to the indicator summary quarto output.
unknown change (overtype or formatting probably) to hospitals summary excel file, but pushing to avoid conflicts :-)
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="285" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{410FC904-7771-4E09-822C-AC205C32145E}"/>
+  <xr:revisionPtr revIDLastSave="286" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D5CC7BB-B862-4B30-8752-48635763011E}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
@@ -1132,152 +1132,152 @@
     </row>
     <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A5" s="17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D5" s="18">
-        <v>40483</v>
+        <v>43344</v>
       </c>
       <c r="E5" s="19">
-        <v>39</v>
-      </c>
-      <c r="F5" s="19">
-        <v>387</v>
+        <v>20</v>
+      </c>
+      <c r="F5" s="22">
+        <v>68</v>
       </c>
       <c r="G5" s="19">
-        <v>387</v>
+        <v>45</v>
       </c>
       <c r="H5" s="19">
-        <v>391</v>
-      </c>
-      <c r="I5" s="17"/>
+        <v>50</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>72</v>
+      </c>
       <c r="J5" s="17" t="s">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="K5" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="L5" s="28" t="s">
-        <v>28</v>
+        <v>14</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A6" s="17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" s="18">
-        <v>43344</v>
-      </c>
-      <c r="E6" s="19">
-        <v>20</v>
-      </c>
-      <c r="F6" s="22">
-        <v>68</v>
-      </c>
-      <c r="G6" s="19">
-        <v>45</v>
-      </c>
-      <c r="H6" s="19">
-        <v>50</v>
+        <v>41760</v>
+      </c>
+      <c r="E6" s="23">
+        <v>95</v>
+      </c>
+      <c r="F6" s="23">
+        <v>1024</v>
+      </c>
+      <c r="G6" s="23">
+        <v>625</v>
+      </c>
+      <c r="H6" s="23">
+        <v>800</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>14</v>
+        <v>75</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="L6" s="17" t="s">
-        <v>59</v>
+        <v>75</v>
+      </c>
+      <c r="L6" s="28" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A7" s="17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D7" s="18">
-        <v>41760</v>
-      </c>
-      <c r="E7" s="23">
-        <v>95</v>
-      </c>
-      <c r="F7" s="23">
-        <v>1024</v>
-      </c>
-      <c r="G7" s="23">
-        <v>625</v>
-      </c>
-      <c r="H7" s="23">
-        <v>800</v>
+        <v>40544</v>
+      </c>
+      <c r="E7" s="19">
+        <v>102</v>
+      </c>
+      <c r="F7" s="19">
+        <v>361</v>
+      </c>
+      <c r="G7" s="19">
+        <v>403</v>
+      </c>
+      <c r="H7" s="19">
+        <v>503</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K7" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L7" s="28" t="s">
-        <v>64</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A8" s="17">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D8" s="18">
-        <v>40544</v>
+        <v>40483</v>
       </c>
       <c r="E8" s="19">
-        <v>102</v>
+        <v>39</v>
       </c>
       <c r="F8" s="19">
-        <v>361</v>
+        <v>387</v>
       </c>
       <c r="G8" s="19">
-        <v>403</v>
+        <v>387</v>
       </c>
       <c r="H8" s="19">
-        <v>503</v>
-      </c>
-      <c r="I8" s="17" t="s">
-        <v>63</v>
-      </c>
+        <v>391</v>
+      </c>
+      <c r="I8" s="17"/>
       <c r="J8" s="17" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L8" s="28" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
@@ -1387,13 +1387,16 @@
       <c r="L12" s="17"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L8">
+    <sortCondition descending="1" ref="D2:D8"/>
+  </sortState>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="L2" r:id="rId1" location=":~:text=The%20old%20hospital%20had%20685,net%20reduction%20of%2014%20beds." xr:uid="{0A92C416-EAF3-4B20-B816-41442BDEC179}"/>
     <hyperlink ref="L3" r:id="rId2" location=":~:text=The%20110%20inpatient%20rooms%20are,for%20patients%20and%20their%20families." display="https://www.clatterbridgecc.nhs.uk/download_file/view/7673/405#:~:text=The%20110%20inpatient%20rooms%20are,for%20patients%20and%20their%20families." xr:uid="{9FB91D32-7B42-4213-8849-B4A3196D6D50}"/>
-    <hyperlink ref="L5" r:id="rId3" xr:uid="{DBE79ACD-2721-4431-B870-B09B6EDE3C2E}"/>
-    <hyperlink ref="L7" r:id="rId4" display="http://www.leaderflushshapland.co.uk/Project-gallery/Southmead-Hospital" xr:uid="{6D8C2DDA-131A-4C54-8996-C8AC29A12373}"/>
-    <hyperlink ref="L8" r:id="rId5" xr:uid="{FD86A662-0C1D-42B1-AC30-1F62B7C9CE88}"/>
+    <hyperlink ref="L8" r:id="rId3" xr:uid="{DBE79ACD-2721-4431-B870-B09B6EDE3C2E}"/>
+    <hyperlink ref="L6" r:id="rId4" display="http://www.leaderflushshapland.co.uk/Project-gallery/Southmead-Hospital" xr:uid="{6D8C2DDA-131A-4C54-8996-C8AC29A12373}"/>
+    <hyperlink ref="L7" r:id="rId5" xr:uid="{FD86A662-0C1D-42B1-AC30-1F62B7C9CE88}"/>
     <hyperlink ref="L9" r:id="rId6" xr:uid="{21A36B13-84D7-4531-9F46-D223B45A17A5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added bibliography link in YAML header, some info on each site in hospital background and updated cells in hospital summary file.
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="290" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D815ABE7-911F-480A-B246-2443AEC98B42}"/>
+  <xr:revisionPtr revIDLastSave="293" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B690C5F6-13F1-4192-BB6F-35930A31059A}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -204,9 +204,6 @@
     <t>ods_code_post</t>
   </si>
   <si>
-    <t>Peterborough (district) Hospital</t>
-  </si>
-  <si>
     <t>Day case and routine inpatient only?</t>
   </si>
   <si>
@@ -271,6 +268,9 @@
   </si>
   <si>
     <t>REN22+REN21</t>
+  </si>
+  <si>
+    <t>Peterborough (city) Hospital</t>
   </si>
 </sst>
 </file>
@@ -971,22 +971,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" customWidth="1"/>
-    <col min="10" max="11" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="164.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="164.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1051,16 +1051,16 @@
       </c>
       <c r="I2" s="17"/>
       <c r="J2" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L2" s="28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1086,19 +1086,19 @@
         <v>89</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J3" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="K3" s="17" t="s">
-        <v>77</v>
-      </c>
       <c r="L3" s="28" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1127,16 +1127,16 @@
         <v>47</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A5" s="17">
         <v>5</v>
       </c>
@@ -1162,19 +1162,19 @@
         <v>50</v>
       </c>
       <c r="I5" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J5" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="K5" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="K5" s="17" t="s">
-        <v>75</v>
-      </c>
       <c r="L5" s="17" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A6" s="17">
         <v>6</v>
       </c>
@@ -1200,19 +1200,19 @@
         <v>800</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A7" s="17">
         <v>7</v>
       </c>
@@ -1238,24 +1238,24 @@
         <v>503</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K7" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L7" s="28" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A8" s="17">
         <v>4</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>9</v>
@@ -1277,16 +1277,16 @@
       </c>
       <c r="I8" s="17"/>
       <c r="J8" s="17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L8" s="28" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H9" s="26"/>
       <c r="I9" s="24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J9" s="24" t="s">
         <v>29</v>
@@ -1320,7 +1320,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -1412,14 +1412,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:P17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="10" width="12.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" customWidth="1"/>
+    <col min="3" max="10" width="12.453125" customWidth="1"/>
+    <col min="13" max="13" width="16.6796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.75">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1445,7 +1445,7 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.75">
       <c r="B2" s="33" t="s">
         <v>42</v>
       </c>
@@ -1463,7 +1463,7 @@
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:16" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:16" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
       <c r="B3" s="34"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
@@ -1493,7 +1493,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B4" s="6" t="s">
         <v>40</v>
       </c>
@@ -1527,9 +1527,9 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B5" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" s="5">
         <v>1</v>
@@ -1564,10 +1564,10 @@
         <v>1</v>
       </c>
       <c r="P5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B6" s="6" t="s">
         <v>39</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B8" s="6" t="s">
         <v>37</v>
       </c>
@@ -1673,7 +1673,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B9" s="6" t="s">
         <v>36</v>
       </c>
@@ -1705,7 +1705,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B10" s="6" t="s">
         <v>35</v>
       </c>
@@ -1737,7 +1737,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B11" s="6" t="s">
         <v>34</v>
       </c>
@@ -1769,9 +1769,9 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B12" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
@@ -1797,7 +1797,7 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B13" s="6" t="s">
         <v>33</v>
       </c>
@@ -1829,7 +1829,7 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B14" s="6" t="s">
         <v>32</v>
       </c>
@@ -1861,7 +1861,7 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="2:16" ht="29.85" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
       <c r="B15" s="3" t="s">
         <v>31</v>
       </c>
@@ -1893,7 +1893,7 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.75">
       <c r="B17" s="30"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sourcing hospitals from excel
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_royalliverpool_newsite/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/anya_ferguson_mlcsu_nhs_uk/Documents/Desktop/nhp_sbr_impacts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="293" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B690C5F6-13F1-4192-BB6F-35930A31059A}"/>
+  <xr:revisionPtr revIDLastSave="323" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6172CFD-DC0B-469C-8147-AC83665AD634}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10965" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="94">
   <si>
     <t>num</t>
   </si>
@@ -271,6 +271,54 @@
   </si>
   <si>
     <t>Peterborough (city) Hospital</t>
+  </si>
+  <si>
+    <t>organisation_code</t>
+  </si>
+  <si>
+    <t>REM</t>
+  </si>
+  <si>
+    <t>REN</t>
+  </si>
+  <si>
+    <t>RGM</t>
+  </si>
+  <si>
+    <t>RAL</t>
+  </si>
+  <si>
+    <t>RVJ</t>
+  </si>
+  <si>
+    <t>RWF</t>
+  </si>
+  <si>
+    <t>RGN</t>
+  </si>
+  <si>
+    <t>site_code</t>
+  </si>
+  <si>
+    <t>REMRQ</t>
+  </si>
+  <si>
+    <t>REN22</t>
+  </si>
+  <si>
+    <t>RGM22</t>
+  </si>
+  <si>
+    <t>RGN80</t>
+  </si>
+  <si>
+    <t>RALC7</t>
+  </si>
+  <si>
+    <t>RVJ01</t>
+  </si>
+  <si>
+    <t>RWFTW</t>
   </si>
 </sst>
 </file>
@@ -651,6 +699,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -970,11 +1022,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
-  <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:O12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.6796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
@@ -983,10 +1035,10 @@
     <col min="8" max="8" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" customWidth="1"/>
     <col min="10" max="11" width="23.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="164.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="164.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1023,8 +1075,14 @@
       <c r="L1" s="17" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M1" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="N1" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1059,8 +1117,14 @@
       <c r="L2" s="28" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M2" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="N2" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1097,8 +1161,14 @@
       <c r="L3" s="28" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M3" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="N3" s="17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1135,8 +1205,14 @@
       <c r="L4" s="17" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M4" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="N4" s="17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="17">
         <v>5</v>
       </c>
@@ -1173,8 +1249,15 @@
       <c r="L5" s="17" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M5" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="N5" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="O5" s="17"/>
+    </row>
+    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="17">
         <v>6</v>
       </c>
@@ -1211,8 +1294,14 @@
       <c r="L6" s="28" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M6" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="N6" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="17">
         <v>7</v>
       </c>
@@ -1249,8 +1338,15 @@
       <c r="L7" s="28" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M7" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="O7" s="17"/>
+    </row>
+    <row r="8" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="17">
         <v>4</v>
       </c>
@@ -1285,8 +1381,15 @@
       <c r="L8" s="28" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" s="27" customFormat="1" ht="16.75" x14ac:dyDescent="0.95">
+      <c r="M8" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="O8" s="17"/>
+    </row>
+    <row r="9" spans="1:15" s="27" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1320,7 +1423,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="10" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1344,7 +1447,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1368,7 +1471,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:12" ht="16.75" x14ac:dyDescent="0.95">
+    <row r="12" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -1412,14 +1515,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A074AA2-DB48-48A9-9A4E-860FBE819769}">
   <dimension ref="B1:P17"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.54296875" customWidth="1"/>
     <col min="3" max="10" width="12.453125" customWidth="1"/>
-    <col min="13" max="13" width="16.6796875" customWidth="1"/>
+    <col min="13" max="13" width="16.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.75">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.35">
       <c r="C1" s="10">
         <v>44835</v>
       </c>
@@ -1445,7 +1548,7 @@
         <v>40483</v>
       </c>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B2" s="33" t="s">
         <v>42</v>
       </c>
@@ -1463,7 +1566,7 @@
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="2:16" s="7" customFormat="1" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:16" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B3" s="34"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
@@ -1493,7 +1596,7 @@
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
     </row>
-    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="6" t="s">
         <v>40</v>
       </c>
@@ -1527,7 +1630,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>65</v>
       </c>
@@ -1567,7 +1670,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="6" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>39</v>
       </c>
@@ -1604,7 +1707,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="7" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>38</v>
       </c>
@@ -1641,7 +1744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="8" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>37</v>
       </c>
@@ -1673,7 +1776,7 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="9" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>36</v>
       </c>
@@ -1705,7 +1808,7 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>35</v>
       </c>
@@ -1737,7 +1840,7 @@
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="11" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>34</v>
       </c>
@@ -1769,7 +1872,7 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="12" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>63</v>
       </c>
@@ -1797,7 +1900,7 @@
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="13" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>33</v>
       </c>
@@ -1829,7 +1932,7 @@
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="14" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>32</v>
       </c>
@@ -1861,7 +1964,7 @@
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="15" spans="2:16" ht="29.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>31</v>
       </c>
@@ -1893,7 +1996,7 @@
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.75">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="30"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding info on type of switch and provider
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/anya_ferguson_mlcsu_nhs_uk/Documents/Desktop/nhp_sbr_impacts/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/anya_ferguson_mlcsu_nhs_uk/Documents/Documents/Files/Projects/nhp_sbr_impacts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6172CFD-DC0B-469C-8147-AC83665AD634}"/>
+  <xr:revisionPtr revIDLastSave="359" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83195440-4E40-4EE1-B03E-6BCB0A6282BD}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="105">
   <si>
     <t>num</t>
   </si>
@@ -319,6 +319,39 @@
   </si>
   <si>
     <t>RWFTW</t>
+  </si>
+  <si>
+    <t>full</t>
+  </si>
+  <si>
+    <t>partial</t>
+  </si>
+  <si>
+    <t>provider</t>
+  </si>
+  <si>
+    <t>Liverpool University Hospitals NHS Foundation Trust</t>
+  </si>
+  <si>
+    <t>The Clatterbridge Cancer Centre NHS Foundation Trust</t>
+  </si>
+  <si>
+    <t>Royal Papworth Hospital NHS Foundation Trust</t>
+  </si>
+  <si>
+    <t>Royal Free London NHS Foundation Trust</t>
+  </si>
+  <si>
+    <t>North Bristol NHS Trust</t>
+  </si>
+  <si>
+    <t>Maidstone and Tunbridge Wells NHS Trust</t>
+  </si>
+  <si>
+    <t>North West Anglia NHS Foundation Trust</t>
+  </si>
+  <si>
+    <t>switch_type</t>
   </si>
 </sst>
 </file>
@@ -1022,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.6328125" bestFit="1" customWidth="1"/>
@@ -1036,9 +1069,10 @@
     <col min="9" max="9" width="39" customWidth="1"/>
     <col min="10" max="11" width="23.08984375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="164.453125" customWidth="1"/>
+    <col min="16" max="16" width="58.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1081,8 +1115,14 @@
       <c r="N1" s="17" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O1" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="P1" s="17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -1123,8 +1163,15 @@
       <c r="N2" s="17" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O2" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="P2" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q2" s="17"/>
+    </row>
+    <row r="3" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -1167,8 +1214,15 @@
       <c r="N3" s="17" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O3" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="P3" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q3" s="17"/>
+    </row>
+    <row r="4" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -1211,8 +1265,15 @@
       <c r="N4" s="17" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O4" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="P4" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q4" s="17"/>
+    </row>
+    <row r="5" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="17">
         <v>5</v>
       </c>
@@ -1255,9 +1316,15 @@
       <c r="N5" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="O5" s="17"/>
-    </row>
-    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O5" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="P5" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q5" s="17"/>
+    </row>
+    <row r="6" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="17">
         <v>6</v>
       </c>
@@ -1300,8 +1367,15 @@
       <c r="N6" s="17" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O6" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="P6" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q6" s="17"/>
+    </row>
+    <row r="7" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="17">
         <v>7</v>
       </c>
@@ -1344,9 +1418,15 @@
       <c r="N7" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="O7" s="17"/>
-    </row>
-    <row r="8" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O7" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="P7" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="Q7" s="17"/>
+    </row>
+    <row r="8" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="17">
         <v>4</v>
       </c>
@@ -1387,9 +1467,15 @@
       <c r="N8" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="O8" s="17"/>
-    </row>
-    <row r="9" spans="1:15" s="27" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="O8" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="P8" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q8" s="17"/>
+    </row>
+    <row r="9" spans="1:17" s="27" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -1423,7 +1509,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -1447,7 +1533,7 @@
       </c>
       <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -1471,7 +1557,7 @@
       </c>
       <c r="L11" s="17"/>
     </row>
-    <row r="12" spans="1:15" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="20">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
hospital summary sheet updated with (some) midlands met info
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/anya_ferguson_mlcsu_nhs_uk/Documents/Documents/Files/Projects/nhp_sbr_impacts/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/NHP/single rooms query/git_repo/nhp_sbr_impacts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="359" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83195440-4E40-4EE1-B03E-6BCB0A6282BD}"/>
+  <xr:revisionPtr revIDLastSave="380" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{868426E3-29CA-4699-AE7E-06FA722BCFAB}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="28680" yWindow="1665" windowWidth="29040" windowHeight="15225" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="112">
   <si>
     <t>num</t>
   </si>
@@ -352,6 +352,27 @@
   </si>
   <si>
     <t>switch_type</t>
+  </si>
+  <si>
+    <t>I3W1A</t>
+  </si>
+  <si>
+    <t>RXK</t>
+  </si>
+  <si>
+    <t>Sandwell and West Birmingham Hospitals NHS Trust</t>
+  </si>
+  <si>
+    <t>Formerly Sandwell and City hospitals. Some IP and OP services remain at those 2 sites.</t>
+  </si>
+  <si>
+    <t>RXK01+RXK02</t>
+  </si>
+  <si>
+    <t>Midlands Metropolitan</t>
+  </si>
+  <si>
+    <t>Smethwick</t>
   </si>
 </sst>
 </file>
@@ -605,7 +626,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -685,6 +706,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -732,10 +754,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1055,11 +1073,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465C2AF7-DCC3-4559-9358-109B6B40D330}">
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
@@ -1580,6 +1598,51 @@
         <v>19</v>
       </c>
       <c r="L12" s="17"/>
+    </row>
+    <row r="13" spans="1:17" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A13" s="20">
+        <v>12</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="35">
+        <v>45566</v>
+      </c>
+      <c r="F13">
+        <f>460+304</f>
+        <v>764</v>
+      </c>
+      <c r="G13">
+        <v>368</v>
+      </c>
+      <c r="H13">
+        <v>736</v>
+      </c>
+      <c r="I13" t="s">
+        <v>108</v>
+      </c>
+      <c r="J13" t="s">
+        <v>109</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="M13" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="O13" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="P13" s="17" t="s">
+        <v>107</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L8">

</xml_diff>

<commit_message>
Update all sql scripts for newest data. Added mid met site info to hospital summary spreadsheet
</commit_message>
<xml_diff>
--- a/hospitals_summary.xlsx
+++ b/hospitals_summary.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="380" documentId="8_{926AE872-106C-4C7C-B02E-ACB99B04BA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{868426E3-29CA-4699-AE7E-06FA722BCFAB}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1665" windowWidth="29040" windowHeight="15225" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
+    <workbookView xWindow="2160" yWindow="2300" windowWidth="14400" windowHeight="7200" xr2:uid="{63CAEA16-0547-4079-B0DF-7240DB91C3F3}"/>
   </bookViews>
   <sheets>
     <sheet name="hospitals" sheetId="1" r:id="rId1"/>
@@ -694,6 +694,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -706,7 +707,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1609,7 +1609,7 @@
       <c r="C13" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D13" s="35">
+      <c r="D13" s="31">
         <v>45566</v>
       </c>
       <c r="F13">
@@ -1698,25 +1698,25 @@
       </c>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="33"/>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
     </row>
     <row r="3" spans="2:16" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B3" s="34"/>
+      <c r="B3" s="35"/>
       <c r="C3" s="9" t="s">
         <v>4</v>
       </c>

</xml_diff>